<commit_message>
Updated HowTo template for Platforms
</commit_message>
<xml_diff>
--- a/public/exportTemplates/platforms.xlsx
+++ b/public/exportTemplates/platforms.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempShare\KYVL_CC_Plus\Export samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41BD3381-2AA6-4410-9DEE-B958FD8EAB23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97722493-8A61-42F0-BA22-6C361F5C0CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13005" yWindow="6300" windowWidth="24645" windowHeight="14385" xr2:uid="{5AA3A021-19FA-4249-BCC4-C0751C521F4C}"/>
+    <workbookView xWindow="5070" yWindow="4635" windowWidth="19905" windowHeight="16965" xr2:uid="{5AA3A021-19FA-4249-BCC4-C0751C521F4C}"/>
   </bookViews>
   <sheets>
     <sheet name="HowToImport" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="58">
   <si>
     <t xml:space="preserve">  * The Platforms tab represents a starting place for updating or importing settings.</t>
   </si>
@@ -69,15 +70,6 @@
     <t xml:space="preserve">  * Columns C-D (Release and Service URL) are required.</t>
   </si>
   <si>
-    <t xml:space="preserve">  * If values are missing or invalid for columns D-N, they will be set to the default.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  * Any header row or columns beyond N will be ignored.</t>
-  </si>
-  <si>
-    <t>COL</t>
-  </si>
-  <si>
     <t>Column Name</t>
   </si>
   <si>
@@ -99,9 +91,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -117,9 +106,6 @@
     <t>If omitted, Platform name used for matching</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -129,15 +115,6 @@
     <t>Platform name</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>5 , 5.1, etc.</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
     <t>Y or N</t>
   </si>
   <si>
@@ -147,9 +124,6 @@
     <t>Y</t>
   </si>
   <si>
-    <t>F</t>
-  </si>
-  <si>
     <t>Harvest Day</t>
   </si>
   <si>
@@ -159,18 +133,12 @@
     <t xml:space="preserve">Day of the month to harvest reports </t>
   </si>
   <si>
-    <t>G</t>
-  </si>
-  <si>
     <t>PR</t>
   </si>
   <si>
     <t>Platform supplies PR reports?</t>
   </si>
   <si>
-    <t>H</t>
-  </si>
-  <si>
     <t>DR</t>
   </si>
   <si>
@@ -180,45 +148,30 @@
     <t>N</t>
   </si>
   <si>
-    <t>I</t>
-  </si>
-  <si>
     <t>TR</t>
   </si>
   <si>
     <t>Platform supplies TR reports?</t>
   </si>
   <si>
-    <t>J</t>
-  </si>
-  <si>
     <t>IR</t>
   </si>
   <si>
     <t>Platform supplies IR reports?</t>
   </si>
   <si>
-    <t>K</t>
-  </si>
-  <si>
     <t>Customer ID</t>
   </si>
   <si>
     <t>Customer ID is required for COUNTER API connections</t>
   </si>
   <si>
-    <t>L</t>
-  </si>
-  <si>
     <t>Requestor ID</t>
   </si>
   <si>
     <t>Requestor ID is required for COUNTER API connections</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
     <t>API Key</t>
   </si>
   <si>
@@ -237,19 +190,37 @@
     <t>Platform Name</t>
   </si>
   <si>
-    <t>COUNTER release(s)  (comma=separated values)</t>
-  </si>
-  <si>
-    <t>COUNTER Releases</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Registry ID</t>
   </si>
   <si>
-    <t>D</t>
+    <t>COUNTER Release</t>
+  </si>
+  <si>
+    <t>COUNTER release</t>
+  </si>
+  <si>
+    <t>Could be 5 ,  5.1,  etc.</t>
+  </si>
+  <si>
+    <t>Refreshable</t>
+  </si>
+  <si>
+    <t>Platform is refreshable from COUNTER registry</t>
+  </si>
+  <si>
+    <t>Service URL</t>
+  </si>
+  <si>
+    <t>COUNTER service URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  * Any header row or columns beyond "O" will be ignored.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  * If values are missing or invalid for columns D-O, they will be set to the default.</t>
   </si>
 </sst>
 </file>
@@ -377,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -388,6 +359,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -406,6 +378,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -711,461 +689,447 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABEB0A5F-61EE-4214-84CD-BA9C82E54CB8}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" customWidth="1"/>
-    <col min="4" max="4" width="51.5703125" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="50.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" customWidth="1"/>
-    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7"/>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="9"/>
-    </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+    <row r="1" spans="1:7" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="10"/>
+    </row>
+    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="12"/>
-    </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="12"/>
-    </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="13"/>
+    </row>
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="12"/>
-    </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="12"/>
-    </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="13"/>
+    </row>
+    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="13"/>
+    </row>
+    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="12"/>
-    </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="13"/>
+    </row>
+    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="16"/>
-    </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="17"/>
+    </row>
+    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="16"/>
-    </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="17"/>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="17"/>
+    </row>
+    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17"/>
+    </row>
+    <row r="12" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="7"/>
+    </row>
+    <row r="13" spans="1:7" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
-    </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="B14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="16"/>
-    </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="6"/>
-    </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="G14" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="1" t="s">
+      <c r="F15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
         <v>15</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="C21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="3" t="s">
+      <c r="F22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F17" s="3" t="s">
+    </row>
+    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G18" s="2" t="s">
+    </row>
+    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G19" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" t="s">
-        <v>25</v>
-      </c>
-      <c r="D20" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G20" s="2" t="s">
+    <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" t="s">
-        <v>25</v>
-      </c>
-      <c r="D21" t="s">
-        <v>42</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G21" s="2" t="s">
+    <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="F29" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C22" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" t="s">
-        <v>46</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23" t="s">
-        <v>48</v>
-      </c>
-      <c r="C23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B24" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" t="s">
-        <v>52</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" t="s">
-        <v>55</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B26" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" t="s">
-        <v>25</v>
-      </c>
-      <c r="D26" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" t="s">
-        <v>25</v>
-      </c>
-      <c r="D27" t="s">
-        <v>60</v>
-      </c>
-      <c r="E27" s="2"/>
-      <c r="G27" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="12">
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:G11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>